<commit_message>
Making code aligned with SoR version2
</commit_message>
<xml_diff>
--- a/Feasibility_and_KPI_results_busplan.xlsx
+++ b/Feasibility_and_KPI_results_busplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\baswe\Documents\GitHub\Project_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280755D0-8274-4C19-9EDF-9DCD78D4D282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5CA002-668F-4747-9927-C7D45171B19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t>Check</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Number of Charging Speeds is equal to 2</t>
+  </si>
+  <si>
+    <t>Assumed SOH percentage between 85% and 95%</t>
   </si>
   <si>
     <t>Battery Capacity at least 10%</t>
@@ -429,10 +432,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="1" max="1" width="39.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -517,10 +520,21 @@
         <v>11</v>
       </c>
       <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
         <v>130</v>
       </c>
-      <c r="C8" t="s">
-        <v>12</v>
+      <c r="C9" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -535,15 +549,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2">
         <v>6537.5404000000044</v>
@@ -551,7 +565,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <v>3533117</v>
@@ -559,7 +573,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4">
         <v>3533.1170000000002</v>
@@ -567,7 +581,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5">
         <v>20</v>
@@ -575,7 +589,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6">
         <v>251</v>
@@ -583,7 +597,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>775</v>
@@ -591,7 +605,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8">
         <v>12.91666666666667</v>
@@ -599,7 +613,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9">
         <v>38.75</v>

</xml_diff>